<commit_message>
add: Adicionado módulo de TMA. Adicionado criação de registros de chamados atendidos no banco.
</commit_message>
<xml_diff>
--- a/df_resumo_atendente.xlsx
+++ b/df_resumo_atendente.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>nome_usuario_incluiu_compra</t>
   </si>
@@ -34,19 +34,7 @@
     <t>index_y</t>
   </si>
   <si>
-    <t>Franciele Pereira Rodrigues</t>
-  </si>
-  <si>
     <t>Rafael Luis Ferreira de Lemos</t>
-  </si>
-  <si>
-    <t>Valquiria Duarte da Silva</t>
-  </si>
-  <si>
-    <t>Compra Maior</t>
-  </si>
-  <si>
-    <t>Compra Menor</t>
   </si>
   <si>
     <t>Compra OK</t>
@@ -410,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -441,19 +429,19 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D2">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>42</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -464,249 +452,19 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D3">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E3">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="F3">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="G3">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="1">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4">
-        <v>54</v>
-      </c>
-      <c r="E4">
-        <v>54</v>
-      </c>
-      <c r="F4">
-        <v>54</v>
-      </c>
-      <c r="G4">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="1">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5">
-        <v>521</v>
-      </c>
-      <c r="E5">
-        <v>521</v>
-      </c>
-      <c r="F5">
-        <v>521</v>
-      </c>
-      <c r="G5">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="1">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6">
-        <v>32</v>
-      </c>
-      <c r="E6">
-        <v>32</v>
-      </c>
-      <c r="F6">
-        <v>32</v>
-      </c>
-      <c r="G6">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7">
-        <v>50</v>
-      </c>
-      <c r="E7">
-        <v>50</v>
-      </c>
-      <c r="F7">
-        <v>50</v>
-      </c>
-      <c r="G7">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="1">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8">
-        <v>51</v>
-      </c>
-      <c r="E8">
-        <v>51</v>
-      </c>
-      <c r="F8">
-        <v>51</v>
-      </c>
-      <c r="G8">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9">
-        <v>129</v>
-      </c>
-      <c r="E9">
-        <v>129</v>
-      </c>
-      <c r="F9">
-        <v>129</v>
-      </c>
-      <c r="G9">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10">
-        <v>20</v>
-      </c>
-      <c r="E10">
-        <v>20</v>
-      </c>
-      <c r="F10">
-        <v>20</v>
-      </c>
-      <c r="G10">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11">
-        <v>41</v>
-      </c>
-      <c r="E11">
-        <v>41</v>
-      </c>
-      <c r="F11">
-        <v>41</v>
-      </c>
-      <c r="G11">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="1">
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12">
-        <v>69</v>
-      </c>
-      <c r="E12">
-        <v>69</v>
-      </c>
-      <c r="F12">
-        <v>69</v>
-      </c>
-      <c r="G12">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="1">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13">
-        <v>460</v>
-      </c>
-      <c r="E13">
-        <v>460</v>
-      </c>
-      <c r="F13">
-        <v>460</v>
-      </c>
-      <c r="G13">
-        <v>460</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified: Ajustado relatório de evolução de precos. Incluido os atendentes da Deep, ajustado a geração dos dados agrupados por filial.
</commit_message>
<xml_diff>
--- a/df_resumo_atendente.xlsx
+++ b/df_resumo_atendente.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="14">
   <si>
     <t>nome_usuario_incluiu_compra</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>Franciele Pereira Rodrigues</t>
+  </si>
+  <si>
+    <t>Larissa de Carvalho Rodrigues</t>
   </si>
   <si>
     <t>Rafael Luis Ferreira de Lemos</t>
@@ -441,19 +444,19 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="E2">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="F2">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="G2">
-        <v>42</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -464,19 +467,19 @@
         <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="E3">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="F3">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="G3">
-        <v>43</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -487,19 +490,19 @@
         <v>6</v>
       </c>
       <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4">
         <v>11</v>
       </c>
-      <c r="D4">
-        <v>54</v>
-      </c>
       <c r="E4">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="F4">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="G4">
-        <v>54</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -510,19 +513,19 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5">
-        <v>521</v>
+        <v>157</v>
       </c>
       <c r="E5">
-        <v>521</v>
+        <v>157</v>
       </c>
       <c r="F5">
-        <v>521</v>
+        <v>157</v>
       </c>
       <c r="G5">
-        <v>521</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -533,19 +536,19 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E6">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="F6">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G6">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -556,19 +559,19 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E7">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>50</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -579,19 +582,19 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="E8">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="F8">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="G8">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -602,19 +605,19 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9">
-        <v>129</v>
+        <v>84</v>
       </c>
       <c r="E9">
-        <v>129</v>
+        <v>84</v>
       </c>
       <c r="F9">
-        <v>129</v>
+        <v>84</v>
       </c>
       <c r="G9">
-        <v>129</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -625,19 +628,19 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D10">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E10">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="F10">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="G10">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -645,22 +648,22 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>
       </c>
       <c r="D11">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="E11">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="F11">
-        <v>41</v>
+        <v>5</v>
       </c>
       <c r="G11">
-        <v>41</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -668,22 +671,22 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="E12">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="F12">
-        <v>69</v>
+        <v>5</v>
       </c>
       <c r="G12">
-        <v>69</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -691,22 +694,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13">
-        <v>460</v>
+        <v>80</v>
       </c>
       <c r="E13">
-        <v>460</v>
+        <v>80</v>
       </c>
       <c r="F13">
-        <v>460</v>
+        <v>80</v>
       </c>
       <c r="G13">
-        <v>460</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: estilização do estilo por empresa.
</commit_message>
<xml_diff>
--- a/df_resumo_atendente.xlsx
+++ b/df_resumo_atendente.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>nome_usuario_incluiu_compra</t>
   </si>
@@ -34,13 +34,19 @@
     <t>index_y</t>
   </si>
   <si>
+    <t>Lucas Fernandes de Oliveira</t>
+  </si>
+  <si>
     <t>Rafael Luis Ferreira de Lemos</t>
   </si>
   <si>
-    <t>Compra OK</t>
+    <t>Valquiria Duarte da Silva</t>
   </si>
   <si>
     <t>Sem Ocorrência</t>
+  </si>
+  <si>
+    <t>Compra Menor</t>
   </si>
 </sst>
 </file>
@@ -398,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -429,19 +435,19 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -449,22 +455,45 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
-      <c r="D3">
-        <v>48</v>
-      </c>
-      <c r="E3">
-        <v>48</v>
-      </c>
-      <c r="F3">
-        <v>48</v>
-      </c>
-      <c r="G3">
-        <v>48</v>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new: plan_controle_fat_2art_terc_app. Implementado justificatica ao estornar pagamento
</commit_message>
<xml_diff>
--- a/df_resumo_atendente.xlsx
+++ b/df_resumo_atendente.xlsx
@@ -14,39 +14,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
   <si>
     <t>nome_usuario_incluiu_compra</t>
   </si>
   <si>
-    <t>status_compra</t>
-  </si>
-  <si>
-    <t>index_x</t>
+    <t>analise</t>
   </si>
   <si>
     <t>qtd_compras</t>
   </si>
   <si>
-    <t>handle_compra_anterior</t>
-  </si>
-  <si>
-    <t>index_y</t>
-  </si>
-  <si>
-    <t>Lucas Fernandes de Oliveira</t>
-  </si>
-  <si>
-    <t>Rafael Luis Ferreira de Lemos</t>
-  </si>
-  <si>
-    <t>Valquiria Duarte da Silva</t>
+    <t>Franciele Pereira Rodrigues</t>
+  </si>
+  <si>
+    <t>Compra Maior</t>
+  </si>
+  <si>
+    <t>Compra Menor</t>
+  </si>
+  <si>
+    <t>Compra OK</t>
   </si>
   <si>
     <t>Sem Ocorrência</t>
-  </si>
-  <si>
-    <t>Compra Menor</t>
   </si>
 </sst>
 </file>
@@ -404,10 +395,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:4">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -417,83 +408,61 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:4">
       <c r="A2" s="1">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
-      </c>
-      <c r="G2">
-        <v>2</v>
+        <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:4">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
+        <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:4">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
suprimentos_evolucao_preco_app. Ajustado a pesquisa por numero de requisição. Ajustado a pesquisa por item. Ajustes na pesquisa informando os filtros obrigatorios
</commit_message>
<xml_diff>
--- a/df_resumo_atendente.xlsx
+++ b/df_resumo_atendente.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="11">
   <si>
     <t>nome_usuario_incluiu_compra</t>
   </si>
@@ -26,6 +26,15 @@
   </si>
   <si>
     <t>Franciele Pereira Rodrigues</t>
+  </si>
+  <si>
+    <t>Larissa de Carvalho Rodrigues</t>
+  </si>
+  <si>
+    <t>Rafael Luis Ferreira de Lemos</t>
+  </si>
+  <si>
+    <t>Valquiria Duarte da Silva</t>
   </si>
   <si>
     <t>Compra Maior</t>
@@ -395,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -417,10 +426,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D2">
-        <v>64</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -431,10 +440,10 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D3">
-        <v>56</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -445,10 +454,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4">
-        <v>80</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -459,10 +468,178 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="1">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="D5">
-        <v>741</v>
+      <c r="D6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="1">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="1">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="1">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="1">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="1">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="1">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="1">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="1">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="1">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17">
+        <v>457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>